<commit_message>
evidence: Q gap A, spot-check report and corrections
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SvqagWL7KU6n6Zjm9yLaNM
</commit_message>
<xml_diff>
--- a/docs/evidence/20261023_Q側缺口_A段/Q側缺口_A段.xlsx
+++ b/docs/evidence/20261023_Q側缺口_A段/Q側缺口_A段.xlsx
@@ -1275,7 +1275,7 @@
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>推論成本（用於毛利率分子）；含免費用戶；是否含 RL／內部使用未明</t>
+          <t>推論成本（用於毛利率分子）；含免費用戶；是否含 RL／內部使用未明。39／45／66 三項細項僅見二手摘要，抽查未能核對</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
@@ -1315,7 +1315,7 @@
       </c>
       <c r="N2" s="4" t="inlineStr">
         <is>
-          <t>口徑：84 億含免費；不含 Microsoft 自家產品推論（Epoch 推定）</t>
+          <t>口徑：84 億含免費；不含 Microsoft 自家產品推論為 Project 預設（Epoch 對 2024 的說法，未證實適用 2025）</t>
         </is>
       </c>
     </row>
@@ -1332,7 +1332,7 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>毛利率 2025 為 33%，低於 2024 的 40% 與內部目標 46%；原因：需求超預期，後期以較貴價格買算力。 / adjusted gross margin 33% vs 40% (2024), target 46%; 'buy more expensive compute at the last minute'.</t>
+          <t>毛利率 2025 為 33%，低於 2024 的 40% 與內部目標 46%；原因（二手摘要的轉述，非逐字引語）：需求超預期，以較貴價格追加算力。 / adjusted gross margin 33% vs 40% (2024), target 46%.</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
@@ -1548,7 +1548,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>某電子報引 The Information：OpenAI「預期去年花 94 億美元於訓練模型的算力」（日期不明，可能為預測）。 / 'expected to spend $9.4 billion on compute for training its AI models last year'.</t>
+          <t>搜尋摘要稱某電子報引 The Information「預期去年花 94 億美元於訓練算力」，抽查找不到該原文；最近可核對者為 2025-09 報導的『2025 訓練逾 90 億』（預測值）。</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -1568,12 +1568,12 @@
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>2025（推定）</t>
+          <t>2025（預測）</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>https://aiafterhours.substack.com/p/openai-vs-anthropic-the-121-billion（搜尋摘要；頁面本環境無法開啟）</t>
+          <t>https://aiafterhours.substack.com/p/openai-vs-anthropic-the-121-billion（搜尋摘要；頁面本環境無法開啟，原文未核對）</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>二手</t>
+          <t>二手（無法核對）</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr">
@@ -1603,7 +1603,7 @@
       </c>
       <c r="N6" s="4" t="inlineStr">
         <is>
-          <t>反駁 120 億：最接近的外部訓練數為 94 億，非 120 億</t>
+          <t>最接近的外部訓練數為約 90–94 億預測，非 120 億；但為預測、未核對原文</t>
         </is>
       </c>
     </row>
@@ -1764,7 +1764,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>The Information（經 The Decoder）：OpenAI 計畫 2026 訓練花 320 億、2027 約 650 億。 / plans to spend $32B on model training in 2026 and ~$65B in 2027.</t>
+          <t>The Information 經 Habr 等二手轉述：OpenAI 計畫 2026 訓練花 320 億、2027 約 650 億（The Decoder 該頁報的是現金燃燒 250／570 億，不是訓練）。 / plans to spend $32B on model training in 2026 and ~$65B in 2027.</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -1799,12 +1799,12 @@
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>二手</t>
+          <t>二手（Habr）；Decoder 頁不支持此數</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="L9" s="4" t="inlineStr">
@@ -1819,7 +1819,7 @@
       </c>
       <c r="N9" s="4" t="inlineStr">
         <is>
-          <t>W4：2026 訓練預測</t>
+          <t>W4：2026 訓練預測（可信度低）</t>
         </is>
       </c>
     </row>
@@ -1836,7 +1836,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>H1 2025 研發費用 67 億（營收 43 億；現金燃燒約 25 億），來自 The Information 對股東文件的報導。 / R&amp;D cost $6.7B in the first half.</t>
+          <t>H1 2025 研發費用 67 億（營收 43 億；現金燃燒約 25 億），僅見 Storyboard18 轉述 The Information（抽查未在 Reuters 找到）。 / R&amp;D cost $6.7B in the first half.</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -1871,12 +1871,12 @@
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>二手（Reuters 轉述）</t>
+          <t>二手（Storyboard18 轉述）</t>
         </is>
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>3–4</t>
         </is>
       </c>
       <c r="L10" s="4" t="inlineStr">
@@ -2124,7 +2124,7 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Oracle：OpenAI 同意每年付 Oracle 約 300 億美元數據中心服務（Oracle 申報：FY2028 起年收入逾 300 億）；容量 4.5 GW。換算 300／4.5＝66.7 億／GW·年；若 5 年 3000 億則 133 億／GW·年。 / agreed to pay Oracle ~$30B a year.</t>
+          <t>Oracle：OpenAI 同意每年付 Oracle 約 300 億美元數據中心服務（Oracle 申報稱 FY2028 起單一合約年收入逾 300 億，申報未點名客戶；OpenAI 與 4.5 GW 來自媒體與 OpenAI 說明）；容量 4.5 GW。換算 300／4.5＝66.7 億／GW·年；若 5 年 3000 億則 133 億／GW·年。 / agreed to pay Oracle ~$30B a year.</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -2412,7 +2412,7 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>AWS：380 億美元、7 年；約 54 億／年；無 MW（『數十萬 GB200／GB300』僅單一部落格）。</t>
+          <t>AWS：380 億美元、7 年；約 54 億／年；無 MW（『數十萬顆 GB200／GB300』為 AWS／OpenAI 公告用語）。</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -2484,7 +2484,7 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Azure 牌價（第三方追蹤站）：ND H100 v5 隨需約 12.29 美元／小時，1 年預留 7.93，3 年預留 5.47；另一站稱承諾折扣上限 1 年 38%、3 年 62%。SKU 是否為每 GPU 價未確認。</t>
+          <t>Azure 牌價（第三方追蹤站）：ND H100 v5 隨需約 12.29 美元／小時，1 年預留 7.93，3 年預留 5.47；價格為每 GPU（8 GPU 實例 98.32÷8＝12.29，已核對）。『38%／62%』折扣上限抽查找不到，且與上列比值不一致，未核對。</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -2509,12 +2509,12 @@
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>https://www.thundercompute.com/blog/azure-gpu-instances（搜尋摘要）</t>
+          <t>https://www.spheron.network/blog/gpu-cloud-pricing-comparison-2026/（搜尋摘要）</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2026-05</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -2529,7 +2529,7 @@
       </c>
       <c r="L19" s="4" t="inlineStr">
         <is>
-          <t>第三方比價站</t>
+          <t>第三方比價站（Spheron）</t>
         </is>
       </c>
       <c r="M19" s="4" t="inlineStr">
@@ -2700,12 +2700,12 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>同口徑長約 ÷ TK（沿用 20261023 持有成本口徑差 B 段）：0.89–1.12。</t>
+          <t>同口徑長約 ÷ TK（沿用 B 段）：證據值 0.89–0.93，另加 Assumed 加價 1.07 得上端 1.12（B 段 build_b.py）；0.89–1.12 為兩者混合區間，非全屬證據。</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>0.89–1.12</t>
+          <t>0.89–0.93（證據）／至 1.12（含 Assumed）</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
@@ -2772,7 +2772,7 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Brockman 法庭證詞：OpenAI 2026 預計算力支出 500 億美元（Reuters 2026-05-05）；報導並稱為 2025 的三倍。 / expects to spend $50 billion on computing power this year.</t>
+          <t>Brockman 法庭證詞：OpenAI 2026 預計算力支出 500 億美元（Reuters 2026-05-05）；（『為 2025 的三倍』一句出自 Epoch，非 Reuters 摘要。） / expects to spend $50 billion on computing power this year.</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
@@ -2844,7 +2844,7 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Epoch 引報導：OpenAI 2025 雲端算力支出 160 億；Brockman『triple what it spent in 2025』→ 隱含 2025 約 167 億，與 160 億一致。</t>
+          <t>Epoch 引報導：OpenAI 2025 雲端算力支出 160 億；Epoch 轉述 Brockman『triple what it spent in 2025』→ 隱含約 167 億。注意：與 W4-01 為同一證詞，非獨立佐證；160 億亦小於審計付 Microsoft 172.1 億（chat 端已查），口徑（雲端算力 vs 付 Microsoft 全部項目）不同。</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">

</xml_diff>

<commit_message>
evidence: Q gap A README per audited accounts (s 0.85-1.0, price 1.5-2.2)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SvqagWL7KU6n6Zjm9yLaNM
</commit_message>
<xml_diff>
--- a/docs/evidence/20261023_Q側缺口_A段/Q側缺口_A段.xlsx
+++ b/docs/evidence/20261023_Q側缺口_A段/Q側缺口_A段.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H45"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -970,7 +970,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>註：口徑因子中檔／高檔取 1/s＝204÷160（Epoch 雲端總支出），為 Derived 且與總支出口徑同源，僅示範量級。</t>
+          <t>註：(d) 為舊版對照，口徑因子取 204÷160（Epoch 雲端總支出）；160 億已被查核帳取代（chat 端），不作結論。</t>
         </is>
       </c>
     </row>
@@ -1144,6 +1144,76 @@
         <v/>
       </c>
       <c r="D45" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="inlineStr">
+        <is>
+          <t>(f) 依查核帳 s（chat 端）反推價格因子 P＝R÷(1/s)＝R×s（必須為真）</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>s（chat 端）</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>P（GW=1.0）</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>P（GW=1.128）</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>P（GW=1.25）</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="B49">
+        <f>$D$17*$A49</f>
+        <v/>
+      </c>
+      <c r="C49">
+        <f>$D$18*$A49</f>
+        <v/>
+      </c>
+      <c r="D49">
+        <f>$D$19*$A49</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B50">
+        <f>$D$17*$A50</f>
+        <v/>
+      </c>
+      <c r="C50">
+        <f>$D$18*$A50</f>
+        <v/>
+      </c>
+      <c r="D50">
+        <f>$D$19*$A50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>chat 端 Derived：Azure 隱含每 GW·年為持有成本的 1.4–2.3 倍（約 $2.3–3.9／GPU 小時），非實付價直接證據</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3667,17 +3737,17 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>口徑因子：204 億（84＋120）超過 Epoch 引的 2025 雲端總支出 160 億，是否要在 B4_Serve 分母改用 160 或 84＋76</t>
+          <t>204 億與 Epoch 160 億的差距，B4_Serve 分母是否調整</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>維持現值 0.41，於報告標註敏感度</t>
+          <t>維持 0.41，160 億已被查核帳取代</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>改動屬判斷類；兩條路對 0.41 的影響請見 README 敏感度</t>
+          <t>查核帳框出 2025 全部算力約 172–210 億，與 204 億相容（s 約 0.85–1.0，chat 端）</t>
         </is>
       </c>
     </row>
@@ -3689,17 +3759,17 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>價格因子是否由 0.85 改採 1.0–1.4 區間</t>
+          <t>價格因子是否由 0.85 改採區間</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>等 chat 端讀 SEC 與 Drive 筆記後定</t>
+          <t>交 chat 端審閱檔</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>本段無 OpenAI 實付 $/GPU·小時</t>
+          <t>本段無 OpenAI 實付價；chat 端 Derived 區間 1.4–2.3 倍</t>
         </is>
       </c>
     </row>

</xml_diff>